<commit_message>
figure 6 for draft 1
</commit_message>
<xml_diff>
--- a/correlations/HI_tauc/HI_tauc_correlations_definitive.xlsx
+++ b/correlations/HI_tauc/HI_tauc_correlations_definitive.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\correlations\HI_tauc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBC3A538-CD0B-49A8-B375-B530CFE371CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFDEEC0A-E801-46A9-A15F-3B05A6F64A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" xr2:uid="{867610DC-2157-4A8B-BAD4-C3624B9432BC}"/>
   </bookViews>
@@ -472,7 +472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -581,13 +581,10 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
@@ -597,17 +594,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,7 +855,7 @@
             <c:numRef>
               <c:f>all!$C$5:$C$20</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="1">
                   <c:v>60.588347259999999</c:v>
@@ -1023,7 +1011,7 @@
             <c:numRef>
               <c:f>all!$C$5:$C$10</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="1">
                   <c:v>60.588347259999999</c:v>
@@ -1170,7 +1158,7 @@
             <c:numRef>
               <c:f>all!$C$11:$C$20</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="2">
                   <c:v>110.72040256</c:v>
@@ -9620,6 +9608,613 @@
       </c:legendEntry>
       <c:legendEntry>
         <c:idx val="5"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>fDOM HI to </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="el-GR" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>τ</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>peak/</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="el-GR" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>τ</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:sysClr>
+                </a:solidFill>
+                <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>c50</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="0"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.0480160568164275E-2"/>
+                  <c:y val="9.3622243457098075E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent6">
+                    <a:lumMod val="20000"/>
+                    <a:lumOff val="80000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>all!$G$61:$G$76</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="1">
+                  <c:v>1.1737788669959504</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.0182769682576838</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0393698938576728</c:v>
+                </c:pt>
+                <c:pt idx="10" formatCode="0.000">
+                  <c:v>1.0331150820718804</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="0.000">
+                  <c:v>1.0275460447393339</c:v>
+                </c:pt>
+                <c:pt idx="12" formatCode="0.000">
+                  <c:v>1.0275826446035865</c:v>
+                </c:pt>
+                <c:pt idx="13" formatCode="0.000">
+                  <c:v>1.0396485920727681</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="0.000">
+                  <c:v>1.0831630031367767</c:v>
+                </c:pt>
+                <c:pt idx="15" formatCode="0.000">
+                  <c:v>1.0183454205725238</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>all!$B$61:$B$76</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>-0.62489073949006502</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-0.54117535564386998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-0.511670862423525</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>-0.22155858359451899</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.6450074853088597E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>-0.24313716774511701</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="0.000">
+                  <c:v>1.3430417175947699E-2</c:v>
+                </c:pt>
+                <c:pt idx="7" formatCode="0.000">
+                  <c:v>-1.61778645652975E-2</c:v>
+                </c:pt>
+                <c:pt idx="8" formatCode="0.000">
+                  <c:v>2.95836818188689E-2</c:v>
+                </c:pt>
+                <c:pt idx="9" formatCode="0.000">
+                  <c:v>-5.4892758010415703E-2</c:v>
+                </c:pt>
+                <c:pt idx="10" formatCode="0.000">
+                  <c:v>8.8641812543785899E-3</c:v>
+                </c:pt>
+                <c:pt idx="11" formatCode="0.000">
+                  <c:v>1.32778322661357E-2</c:v>
+                </c:pt>
+                <c:pt idx="12" formatCode="0.000">
+                  <c:v>-6.0975544853349099E-2</c:v>
+                </c:pt>
+                <c:pt idx="13" formatCode="0.000">
+                  <c:v>-1.77749404385871E-2</c:v>
+                </c:pt>
+                <c:pt idx="14" formatCode="0.000">
+                  <c:v>3.08855730575289E-3</c:v>
+                </c:pt>
+                <c:pt idx="15" formatCode="0.000">
+                  <c:v>-5.3081166180475401E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-51B7-4E42-9079-86E703A7E016}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="482930495"/>
+        <c:axId val="482950655"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="482930495"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="482950655"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="482950655"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="el-GR">
+                    <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>τ</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US">
+                    <a:latin typeface="Aptos" panose="020B0004020202020204" pitchFamily="34" charset="0"/>
+                  </a:rPr>
+                  <a:t>c50</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="482930495"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="1"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:overlay val="0"/>
@@ -15487,10 +16082,10 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.1737788669959499</c:v>
+                  <c:v>1.1737788669959504</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.01827696825768</c:v>
+                  <c:v>1.0182769682576838</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1</c:v>
@@ -15499,22 +16094,22 @@
                   <c:v>1.0393698938576728</c:v>
                 </c:pt>
                 <c:pt idx="9" formatCode="0.000">
-                  <c:v>1.0311456359907301</c:v>
+                  <c:v>1.0331150820718804</c:v>
                 </c:pt>
                 <c:pt idx="10" formatCode="0.000">
-                  <c:v>1.0328896319418399</c:v>
+                  <c:v>1.0275460447393339</c:v>
                 </c:pt>
                 <c:pt idx="11" formatCode="0.000">
-                  <c:v>1.0327006459464001</c:v>
+                  <c:v>1.0275826446035865</c:v>
                 </c:pt>
                 <c:pt idx="12" formatCode="0.000">
-                  <c:v>1.06939420314209</c:v>
+                  <c:v>1.0396485920727681</c:v>
                 </c:pt>
                 <c:pt idx="13" formatCode="0.000">
-                  <c:v>1.12591121276406</c:v>
+                  <c:v>1.0831630031367767</c:v>
                 </c:pt>
                 <c:pt idx="14" formatCode="0.000">
-                  <c:v>1.06457347177821</c:v>
+                  <c:v>1.0183454205725238</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -15527,134 +16122,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="1"/>
           <c:order val="1"/>
-          <c:tx>
-            <c:v>summer</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="0"/>
-            <c:trendlineLbl>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:solidFill>
-                  <a:schemeClr val="tx2">
-                    <a:lumMod val="10000"/>
-                    <a:lumOff val="90000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>all!$B$62:$B$66</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>-0.54117535564386998</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>-0.511670862423525</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-0.22155858359451899</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>9.6450074853088597E-2</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>-0.24313716774511701</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>all!$G$62:$G$66</c:f>
-              <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>1.1737788669959499</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.01827696825768</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3C41-49CB-B36C-8321121D3231}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="2"/>
           <c:tx>
             <c:v>spring</c:v>
           </c:tx>
@@ -15784,22 +16253,22 @@
                   <c:v>1.0393698938576728</c:v>
                 </c:pt>
                 <c:pt idx="4" formatCode="0.000">
-                  <c:v>1.0311456359907301</c:v>
+                  <c:v>1.0331150820718804</c:v>
                 </c:pt>
                 <c:pt idx="5" formatCode="0.000">
-                  <c:v>1.0328896319418399</c:v>
+                  <c:v>1.0275460447393339</c:v>
                 </c:pt>
                 <c:pt idx="6" formatCode="0.000">
-                  <c:v>1.0327006459464001</c:v>
+                  <c:v>1.0275826446035865</c:v>
                 </c:pt>
                 <c:pt idx="7" formatCode="0.000">
-                  <c:v>1.06939420314209</c:v>
+                  <c:v>1.0396485920727681</c:v>
                 </c:pt>
                 <c:pt idx="8" formatCode="0.000">
-                  <c:v>1.12591121276406</c:v>
+                  <c:v>1.0831630031367767</c:v>
                 </c:pt>
                 <c:pt idx="9" formatCode="0.000">
-                  <c:v>1.06457347177821</c:v>
+                  <c:v>1.0183454205725238</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -16077,15 +16546,11 @@
     <c:legend>
       <c:legendPos val="b"/>
       <c:legendEntry>
-        <c:idx val="3"/>
+        <c:idx val="2"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:legendEntry>
-        <c:idx val="4"/>
-        <c:delete val="1"/>
-      </c:legendEntry>
-      <c:legendEntry>
-        <c:idx val="5"/>
+        <c:idx val="3"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:overlay val="0"/>
@@ -17495,6 +17960,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors19.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -22460,6 +22965,522 @@
 </file>
 
 <file path=xl/charts/style18.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style19.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -27787,6 +28808,44 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>616324</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>134471</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7080980F-DF29-4665-AD45-A3C8CCF24535}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -28196,7 +29255,7 @@
       <c r="I4" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="54" t="s">
+      <c r="J4" s="37" t="s">
         <v>64</v>
       </c>
       <c r="K4" s="3"/>
@@ -28246,7 +29305,7 @@
       <c r="G5" s="18"/>
       <c r="H5" s="25"/>
       <c r="I5" s="15"/>
-      <c r="J5" s="55"/>
+      <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
@@ -28285,7 +29344,7 @@
       <c r="B6" s="16">
         <v>0.17369777575697301</v>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <v>60.588347259999999</v>
       </c>
       <c r="D6" s="19">
@@ -28348,7 +29407,7 @@
       <c r="B7" s="16">
         <v>9.9143945152060597E-2</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="18">
         <v>73.387016439999996</v>
       </c>
       <c r="D7" s="19">
@@ -28411,7 +29470,7 @@
       <c r="B8" s="16">
         <v>0.21234239309632399</v>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="18">
         <v>79.767295559999994</v>
       </c>
       <c r="D8" s="19">
@@ -28474,7 +29533,7 @@
       <c r="B9" s="16">
         <v>0.36516163611226798</v>
       </c>
-      <c r="C9" s="17"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="19">
         <v>365</v>
       </c>
@@ -28485,7 +29544,7 @@
       <c r="G9" s="18"/>
       <c r="H9" s="18"/>
       <c r="I9" s="18"/>
-      <c r="J9" s="56"/>
+      <c r="J9" s="9"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
@@ -28524,7 +29583,7 @@
       <c r="B10" s="16">
         <v>4.1333778886518201E-2</v>
       </c>
-      <c r="C10" s="17"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="19">
         <v>351.5</v>
       </c>
@@ -28535,7 +29594,7 @@
       <c r="G10" s="18"/>
       <c r="H10" s="18"/>
       <c r="I10" s="18"/>
-      <c r="J10" s="56"/>
+      <c r="J10" s="9"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
@@ -28574,7 +29633,7 @@
       <c r="B11" s="16">
         <v>9.4513218106104094E-2</v>
       </c>
-      <c r="C11" s="20"/>
+      <c r="C11" s="50"/>
       <c r="D11" s="19"/>
       <c r="E11" s="19"/>
       <c r="F11" s="18">
@@ -28583,7 +29642,7 @@
       <c r="G11" s="18"/>
       <c r="H11" s="18"/>
       <c r="I11" s="18"/>
-      <c r="J11" s="56"/>
+      <c r="J11" s="9"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
@@ -28622,7 +29681,7 @@
       <c r="B12" s="16">
         <v>4.2663094228711902E-2</v>
       </c>
-      <c r="C12" s="20"/>
+      <c r="C12" s="50"/>
       <c r="D12" s="19">
         <v>22</v>
       </c>
@@ -28633,7 +29692,7 @@
       <c r="G12" s="18"/>
       <c r="H12" s="18"/>
       <c r="I12" s="18"/>
-      <c r="J12" s="56"/>
+      <c r="J12" s="9"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
@@ -28672,7 +29731,7 @@
       <c r="B13" s="16">
         <v>8.8732929175135894E-2</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="18">
         <v>110.72040256</v>
       </c>
       <c r="D13" s="19">
@@ -28735,7 +29794,7 @@
       <c r="B14" s="16">
         <v>-1.9463558010346702E-2</v>
       </c>
-      <c r="C14" s="17"/>
+      <c r="C14" s="18"/>
       <c r="D14" s="19">
         <v>21.5</v>
       </c>
@@ -28746,7 +29805,7 @@
       <c r="G14" s="18"/>
       <c r="H14" s="18"/>
       <c r="I14" s="18"/>
-      <c r="J14" s="56"/>
+      <c r="J14" s="9"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -28785,7 +29844,7 @@
       <c r="B15" s="16">
         <v>0.10415722716452799</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="18">
         <v>111.66319882000001</v>
       </c>
       <c r="D15" s="19">
@@ -28821,7 +29880,7 @@
       <c r="B16" s="16">
         <v>4.66251429291673E-2</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="18">
         <v>114.89097618</v>
       </c>
       <c r="D16" s="19">
@@ -28857,7 +29916,7 @@
       <c r="B17" s="16">
         <v>9.0894558490112708E-3</v>
       </c>
-      <c r="C17" s="17">
+      <c r="C17" s="18">
         <v>116.55531655999999</v>
       </c>
       <c r="D17" s="19">
@@ -28893,7 +29952,7 @@
       <c r="B18" s="16">
         <v>-1.7278096303121701E-2</v>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="18">
         <v>120.40602251999999</v>
       </c>
       <c r="D18" s="19">
@@ -28929,7 +29988,7 @@
       <c r="B19" s="16">
         <v>2.0373962034653699E-2</v>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="18">
         <v>118.75512236</v>
       </c>
       <c r="D19" s="19">
@@ -28942,7 +30001,7 @@
         <v>128.631154973333</v>
       </c>
       <c r="G19" s="18">
-        <f t="shared" si="0"/>
+        <f>F19/C19</f>
         <v>1.0831630031367767</v>
       </c>
       <c r="H19" s="18">
@@ -28987,7 +30046,7 @@
       <c r="B20" s="16">
         <v>-2.50118292734785E-2</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="18">
         <v>125.12197168</v>
       </c>
       <c r="D20" s="19">
@@ -29050,10 +30109,10 @@
       <c r="K21" s="8"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
-      <c r="V21" s="40" t="s">
+      <c r="V21" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="W21" s="42">
+      <c r="W21" s="41">
         <v>0.76444358594083117</v>
       </c>
       <c r="X21" s="27"/>
@@ -29067,7 +30126,7 @@
       <c r="AF21" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="AG21" s="44">
+      <c r="AG21" s="41">
         <v>0.61098104839357625</v>
       </c>
       <c r="AH21" s="30"/>
@@ -29093,10 +30152,10 @@
       <c r="J22" s="6"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
-      <c r="V22" s="40" t="s">
+      <c r="V22" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="W22" s="42">
+      <c r="W22" s="41">
         <v>0.58437399608607699</v>
       </c>
       <c r="X22" s="27"/>
@@ -29110,7 +30169,7 @@
       <c r="AF22" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="AG22" s="44">
+      <c r="AG22" s="41">
         <v>0.373297841496114</v>
       </c>
       <c r="AH22" s="30"/>
@@ -29149,14 +30208,14 @@
       <c r="I23" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="J23" s="54"/>
+      <c r="J23" s="37"/>
       <c r="K23" s="8"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
-      <c r="V23" s="40" t="s">
+      <c r="V23" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="W23" s="42">
+      <c r="W23" s="41">
         <v>0.46562370925352753</v>
       </c>
       <c r="X23" s="27"/>
@@ -29170,7 +30229,7 @@
       <c r="AF23" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="AG23" s="44">
+      <c r="AG23" s="41">
         <v>0.19424008192357453</v>
       </c>
       <c r="AH23" s="30"/>
@@ -29197,14 +30256,14 @@
       <c r="G24" s="18"/>
       <c r="H24" s="25"/>
       <c r="I24" s="15"/>
-      <c r="J24" s="55"/>
+      <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
-      <c r="V24" s="40" t="s">
+      <c r="V24" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="W24" s="40">
+      <c r="W24" s="27">
         <v>5.8038237190838761E-2</v>
       </c>
       <c r="X24" s="27"/>
@@ -29218,7 +30277,7 @@
       <c r="AF24" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="AG24" s="44">
+      <c r="AG24" s="41">
         <v>0.16038868504292825</v>
       </c>
       <c r="AH24" s="30"/>
@@ -29263,10 +30322,10 @@
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
-      <c r="V25" s="41" t="s">
+      <c r="V25" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="W25" s="41">
+      <c r="W25" s="40">
         <v>10</v>
       </c>
       <c r="X25" s="27"/>
@@ -29421,7 +30480,7 @@
       <c r="G28" s="18"/>
       <c r="H28" s="18"/>
       <c r="I28" s="18"/>
-      <c r="J28" s="56"/>
+      <c r="J28" s="9"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -29483,26 +30542,26 @@
       <c r="G29" s="18"/>
       <c r="H29" s="18"/>
       <c r="I29" s="18"/>
-      <c r="J29" s="56"/>
+      <c r="J29" s="9"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
-      <c r="V29" s="40" t="s">
+      <c r="V29" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="W29" s="40">
+      <c r="W29" s="27">
         <v>2</v>
       </c>
-      <c r="X29" s="40">
+      <c r="X29" s="27">
         <v>3.315237426135248E-2</v>
       </c>
-      <c r="Y29" s="40">
+      <c r="Y29" s="27">
         <v>1.657618713067624E-2</v>
       </c>
-      <c r="Z29" s="40">
+      <c r="Z29" s="27">
         <v>4.9210322911481184</v>
       </c>
-      <c r="AA29" s="40">
+      <c r="AA29" s="27">
         <v>4.6287048710281858E-2</v>
       </c>
       <c r="AB29" s="27"/>
@@ -29549,24 +30608,24 @@
       <c r="G30" s="18"/>
       <c r="H30" s="18"/>
       <c r="I30" s="18"/>
-      <c r="J30" s="56"/>
+      <c r="J30" s="9"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
-      <c r="V30" s="40" t="s">
+      <c r="V30" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="W30" s="40">
+      <c r="W30" s="27">
         <v>7</v>
       </c>
-      <c r="X30" s="40">
+      <c r="X30" s="27">
         <v>2.3579058833540417E-2</v>
       </c>
-      <c r="Y30" s="40">
+      <c r="Y30" s="27">
         <v>3.3684369762200595E-3</v>
       </c>
-      <c r="Z30" s="40"/>
-      <c r="AA30" s="40"/>
+      <c r="Z30" s="27"/>
+      <c r="AA30" s="27"/>
       <c r="AB30" s="27"/>
       <c r="AC30" s="27"/>
       <c r="AD30" s="27"/>
@@ -29607,22 +30666,22 @@
       <c r="G31" s="18"/>
       <c r="H31" s="18"/>
       <c r="I31" s="18"/>
-      <c r="J31" s="56"/>
+      <c r="J31" s="9"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
-      <c r="V31" s="41" t="s">
+      <c r="V31" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="W31" s="41">
+      <c r="W31" s="40">
         <v>9</v>
       </c>
-      <c r="X31" s="41">
+      <c r="X31" s="40">
         <v>5.6731433094892897E-2</v>
       </c>
-      <c r="Y31" s="41"/>
-      <c r="Z31" s="41"/>
-      <c r="AA31" s="41"/>
+      <c r="Y31" s="40"/>
+      <c r="Z31" s="40"/>
+      <c r="AA31" s="40"/>
       <c r="AB31" s="27"/>
       <c r="AC31" s="27"/>
       <c r="AD31" s="27"/>
@@ -29716,7 +30775,7 @@
       <c r="G33" s="18"/>
       <c r="H33" s="18"/>
       <c r="I33" s="18"/>
-      <c r="J33" s="56"/>
+      <c r="J33" s="9"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -29792,7 +30851,7 @@
         <v>115.360934813333</v>
       </c>
       <c r="G34" s="18">
-        <f t="shared" ref="G33:G39" si="1">F34/C34</f>
+        <f t="shared" ref="G34:G39" si="1">F34/C34</f>
         <v>1.0331150820718804</v>
       </c>
       <c r="H34" s="18">
@@ -29807,31 +30866,31 @@
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
-      <c r="V34" s="40" t="s">
+      <c r="V34" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="W34" s="40">
+      <c r="W34" s="27">
         <v>-0.10711095089458646</v>
       </c>
-      <c r="X34" s="40">
+      <c r="X34" s="27">
         <v>0.41296001163183188</v>
       </c>
-      <c r="Y34" s="40">
+      <c r="Y34" s="27">
         <v>-0.25937366301238768</v>
       </c>
-      <c r="Z34" s="42">
+      <c r="Z34" s="41">
         <v>0.80280949286419134</v>
       </c>
-      <c r="AA34" s="40">
+      <c r="AA34" s="27">
         <v>-1.0836062093372547</v>
       </c>
-      <c r="AB34" s="40">
+      <c r="AB34" s="27">
         <v>0.86938430754808171</v>
       </c>
-      <c r="AC34" s="40">
+      <c r="AC34" s="27">
         <v>-1.0836062093372547</v>
       </c>
-      <c r="AD34" s="40">
+      <c r="AD34" s="27">
         <v>0.86938430754808171</v>
       </c>
       <c r="AE34" s="1"/>
@@ -29847,7 +30906,7 @@
       <c r="AI34" s="30">
         <v>-1.1263311316356921</v>
       </c>
-      <c r="AJ34" s="44">
+      <c r="AJ34" s="41">
         <v>0.29715241337808557</v>
       </c>
       <c r="AK34" s="30">
@@ -29898,31 +30957,31 @@
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
-      <c r="V35" s="40" t="s">
+      <c r="V35" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="W35" s="40">
+      <c r="W35" s="27">
         <v>0.24640880866478085</v>
       </c>
-      <c r="X35" s="40">
+      <c r="X35" s="27">
         <v>0.39090774190003369</v>
       </c>
-      <c r="Y35" s="40">
+      <c r="Y35" s="27">
         <v>0.63035029049845381</v>
       </c>
-      <c r="Z35" s="42">
+      <c r="Z35" s="41">
         <v>0.54848269619738965</v>
       </c>
-      <c r="AA35" s="40">
+      <c r="AA35" s="27">
         <v>-0.67794111796741185</v>
       </c>
-      <c r="AB35" s="40">
+      <c r="AB35" s="27">
         <v>1.1707587352969735</v>
       </c>
-      <c r="AC35" s="40">
+      <c r="AC35" s="27">
         <v>-0.67794111796741185</v>
       </c>
-      <c r="AD35" s="40">
+      <c r="AD35" s="27">
         <v>1.1707587352969735</v>
       </c>
       <c r="AE35" s="1"/>
@@ -29938,7 +30997,7 @@
       <c r="AI35" s="30">
         <v>0.94119383587194227</v>
       </c>
-      <c r="AJ35" s="44">
+      <c r="AJ35" s="41">
         <v>0.3779426283901085</v>
       </c>
       <c r="AK35" s="30">
@@ -29989,31 +31048,31 @@
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
-      <c r="V36" s="41" t="s">
+      <c r="V36" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="W36" s="41">
+      <c r="W36" s="40">
         <v>1.6496532218056408E-2</v>
       </c>
-      <c r="X36" s="41">
+      <c r="X36" s="40">
         <v>5.5166414100202782E-3</v>
       </c>
-      <c r="Y36" s="41">
+      <c r="Y36" s="40">
         <v>2.9903216453570014</v>
       </c>
-      <c r="Z36" s="43">
+      <c r="Z36" s="42">
         <v>2.0217138054056741E-2</v>
       </c>
-      <c r="AA36" s="41">
+      <c r="AA36" s="40">
         <v>3.4517481525814415E-3</v>
       </c>
-      <c r="AB36" s="41">
+      <c r="AB36" s="40">
         <v>2.9541316283531373E-2</v>
       </c>
-      <c r="AC36" s="41">
+      <c r="AC36" s="40">
         <v>3.4517481525814415E-3</v>
       </c>
-      <c r="AD36" s="41">
+      <c r="AD36" s="40">
         <v>2.9541316283531373E-2</v>
       </c>
       <c r="AE36" s="1"/>
@@ -30029,7 +31088,7 @@
       <c r="AI36" s="32">
         <v>-1.731321476916527</v>
       </c>
-      <c r="AJ36" s="52">
+      <c r="AJ36" s="42">
         <v>0.12700526854237526</v>
       </c>
       <c r="AK36" s="32">
@@ -30129,15 +31188,15 @@
       <c r="AC38" s="35"/>
       <c r="AD38" s="35"/>
       <c r="AE38" s="1"/>
-      <c r="AF38" s="47"/>
-      <c r="AG38" s="47"/>
-      <c r="AH38" s="47"/>
-      <c r="AI38" s="47"/>
-      <c r="AJ38" s="47"/>
-      <c r="AK38" s="47"/>
-      <c r="AL38" s="47"/>
-      <c r="AM38" s="47"/>
-      <c r="AN38" s="47"/>
+      <c r="AF38" s="44"/>
+      <c r="AG38" s="44"/>
+      <c r="AH38" s="44"/>
+      <c r="AI38" s="44"/>
+      <c r="AJ38" s="44"/>
+      <c r="AK38" s="44"/>
+      <c r="AL38" s="44"/>
+      <c r="AM38" s="44"/>
+      <c r="AN38" s="44"/>
     </row>
     <row r="39" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
@@ -30186,26 +31245,26 @@
       <c r="AC39" s="35"/>
       <c r="AD39" s="35"/>
       <c r="AE39" s="1"/>
-      <c r="AF39" s="48" t="s">
+      <c r="AF39" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="AG39" s="48"/>
-      <c r="AH39" s="47"/>
-      <c r="AI39" s="47"/>
-      <c r="AJ39" s="47"/>
-      <c r="AK39" s="47"/>
-      <c r="AL39" s="47"/>
-      <c r="AM39" s="47"/>
-      <c r="AN39" s="47"/>
+      <c r="AG39" s="45"/>
+      <c r="AH39" s="44"/>
+      <c r="AI39" s="44"/>
+      <c r="AJ39" s="44"/>
+      <c r="AK39" s="44"/>
+      <c r="AL39" s="44"/>
+      <c r="AM39" s="44"/>
+      <c r="AN39" s="44"/>
     </row>
     <row r="40" spans="1:40" x14ac:dyDescent="0.25">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
-      <c r="V40" s="45" t="s">
+      <c r="V40" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="W40" s="42">
+      <c r="W40" s="41">
         <v>0.72180686146740602</v>
       </c>
       <c r="X40" s="35"/>
@@ -30216,19 +31275,19 @@
       <c r="AC40" s="35"/>
       <c r="AD40" s="35"/>
       <c r="AE40" s="1"/>
-      <c r="AF40" s="47" t="s">
+      <c r="AF40" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="AG40" s="51">
+      <c r="AG40" s="48">
         <v>0.81667320319882508</v>
       </c>
-      <c r="AH40" s="47"/>
-      <c r="AI40" s="47"/>
-      <c r="AJ40" s="47"/>
-      <c r="AK40" s="47"/>
-      <c r="AL40" s="47"/>
-      <c r="AM40" s="47"/>
-      <c r="AN40" s="47"/>
+      <c r="AH40" s="44"/>
+      <c r="AI40" s="44"/>
+      <c r="AJ40" s="44"/>
+      <c r="AK40" s="44"/>
+      <c r="AL40" s="44"/>
+      <c r="AM40" s="44"/>
+      <c r="AN40" s="44"/>
     </row>
     <row r="41" spans="1:40" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
@@ -30258,14 +31317,14 @@
       <c r="I41" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="J41" s="54"/>
+      <c r="J41" s="37"/>
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
-      <c r="V41" s="45" t="s">
+      <c r="V41" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="W41" s="42">
+      <c r="W41" s="41">
         <v>0.52100514526142705</v>
       </c>
       <c r="X41" s="35"/>
@@ -30276,19 +31335,19 @@
       <c r="AC41" s="35"/>
       <c r="AD41" s="35"/>
       <c r="AE41" s="1"/>
-      <c r="AF41" s="47" t="s">
+      <c r="AF41" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="AG41" s="51">
+      <c r="AG41" s="48">
         <v>0.66695512082302943</v>
       </c>
-      <c r="AH41" s="47"/>
-      <c r="AI41" s="47"/>
-      <c r="AJ41" s="47"/>
-      <c r="AK41" s="47"/>
-      <c r="AL41" s="47"/>
-      <c r="AM41" s="47"/>
-      <c r="AN41" s="47"/>
+      <c r="AH41" s="44"/>
+      <c r="AI41" s="44"/>
+      <c r="AJ41" s="44"/>
+      <c r="AK41" s="44"/>
+      <c r="AL41" s="44"/>
+      <c r="AM41" s="44"/>
+      <c r="AN41" s="44"/>
     </row>
     <row r="42" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
@@ -30306,14 +31365,14 @@
       <c r="G42" s="18"/>
       <c r="H42" s="25"/>
       <c r="I42" s="15"/>
-      <c r="J42" s="55"/>
+      <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
-      <c r="V42" s="45" t="s">
+      <c r="V42" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="W42" s="42">
+      <c r="W42" s="41">
         <v>0.38414947247897757</v>
       </c>
       <c r="X42" s="35"/>
@@ -30324,19 +31383,19 @@
       <c r="AC42" s="35"/>
       <c r="AD42" s="35"/>
       <c r="AE42" s="1"/>
-      <c r="AF42" s="47" t="s">
+      <c r="AF42" s="44" t="s">
         <v>41</v>
       </c>
-      <c r="AG42" s="51">
+      <c r="AG42" s="48">
         <v>0.5717994410581807</v>
       </c>
-      <c r="AH42" s="47"/>
-      <c r="AI42" s="47"/>
-      <c r="AJ42" s="47"/>
-      <c r="AK42" s="47"/>
-      <c r="AL42" s="47"/>
-      <c r="AM42" s="47"/>
-      <c r="AN42" s="47"/>
+      <c r="AH42" s="44"/>
+      <c r="AI42" s="44"/>
+      <c r="AJ42" s="44"/>
+      <c r="AK42" s="44"/>
+      <c r="AL42" s="44"/>
+      <c r="AM42" s="44"/>
+      <c r="AN42" s="44"/>
     </row>
     <row r="43" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A43" s="15" t="s">
@@ -30372,10 +31431,10 @@
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
-      <c r="V43" s="45" t="s">
+      <c r="V43" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="W43" s="45">
+      <c r="W43" s="35">
         <v>3.6966086835203485E-2</v>
       </c>
       <c r="X43" s="35"/>
@@ -30386,19 +31445,19 @@
       <c r="AC43" s="35"/>
       <c r="AD43" s="35"/>
       <c r="AE43" s="1"/>
-      <c r="AF43" s="47" t="s">
+      <c r="AF43" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="AG43" s="47">
+      <c r="AG43" s="44">
         <v>0.1445251291895934</v>
       </c>
-      <c r="AH43" s="47"/>
-      <c r="AI43" s="47"/>
-      <c r="AJ43" s="47"/>
-      <c r="AK43" s="47"/>
-      <c r="AL43" s="47"/>
-      <c r="AM43" s="47"/>
-      <c r="AN43" s="47"/>
+      <c r="AH43" s="44"/>
+      <c r="AI43" s="44"/>
+      <c r="AJ43" s="44"/>
+      <c r="AK43" s="44"/>
+      <c r="AL43" s="44"/>
+      <c r="AM43" s="44"/>
+      <c r="AN43" s="44"/>
     </row>
     <row r="44" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="15" t="s">
@@ -30441,10 +31500,10 @@
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
       <c r="T44" s="1"/>
-      <c r="V44" s="46" t="s">
+      <c r="V44" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="W44" s="46">
+      <c r="W44" s="43">
         <v>10</v>
       </c>
       <c r="X44" s="35"/>
@@ -30455,19 +31514,19 @@
       <c r="AC44" s="35"/>
       <c r="AD44" s="35"/>
       <c r="AE44" s="1"/>
-      <c r="AF44" s="49" t="s">
+      <c r="AF44" s="46" t="s">
         <v>43</v>
       </c>
-      <c r="AG44" s="49">
+      <c r="AG44" s="46">
         <v>10</v>
       </c>
-      <c r="AH44" s="47"/>
-      <c r="AI44" s="47"/>
-      <c r="AJ44" s="47"/>
-      <c r="AK44" s="47"/>
-      <c r="AL44" s="47"/>
-      <c r="AM44" s="47"/>
-      <c r="AN44" s="47"/>
+      <c r="AH44" s="44"/>
+      <c r="AI44" s="44"/>
+      <c r="AJ44" s="44"/>
+      <c r="AK44" s="44"/>
+      <c r="AL44" s="44"/>
+      <c r="AM44" s="44"/>
+      <c r="AN44" s="44"/>
     </row>
     <row r="45" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
@@ -30513,15 +31572,15 @@
       <c r="AC45" s="35"/>
       <c r="AD45" s="35"/>
       <c r="AE45" s="1"/>
-      <c r="AF45" s="47"/>
-      <c r="AG45" s="47"/>
-      <c r="AH45" s="47"/>
-      <c r="AI45" s="47"/>
-      <c r="AJ45" s="47"/>
-      <c r="AK45" s="47"/>
-      <c r="AL45" s="47"/>
-      <c r="AM45" s="47"/>
-      <c r="AN45" s="47"/>
+      <c r="AF45" s="44"/>
+      <c r="AG45" s="44"/>
+      <c r="AH45" s="44"/>
+      <c r="AI45" s="44"/>
+      <c r="AJ45" s="44"/>
+      <c r="AK45" s="44"/>
+      <c r="AL45" s="44"/>
+      <c r="AM45" s="44"/>
+      <c r="AN45" s="44"/>
     </row>
     <row r="46" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="15" t="s">
@@ -30541,7 +31600,7 @@
       <c r="G46" s="18"/>
       <c r="H46" s="18"/>
       <c r="I46" s="18"/>
-      <c r="J46" s="56"/>
+      <c r="J46" s="9"/>
       <c r="L46" s="2"/>
       <c r="M46" s="1"/>
       <c r="T46" s="1"/>
@@ -30556,17 +31615,17 @@
       <c r="AB46" s="35"/>
       <c r="AC46" s="35"/>
       <c r="AD46" s="35"/>
-      <c r="AF46" s="47" t="s">
+      <c r="AF46" s="44" t="s">
         <v>44</v>
       </c>
-      <c r="AG46" s="47"/>
-      <c r="AH46" s="47"/>
-      <c r="AI46" s="47"/>
-      <c r="AJ46" s="47"/>
-      <c r="AK46" s="47"/>
-      <c r="AL46" s="47"/>
-      <c r="AM46" s="47"/>
-      <c r="AN46" s="47"/>
+      <c r="AG46" s="44"/>
+      <c r="AH46" s="44"/>
+      <c r="AI46" s="44"/>
+      <c r="AJ46" s="44"/>
+      <c r="AK46" s="44"/>
+      <c r="AL46" s="44"/>
+      <c r="AM46" s="44"/>
+      <c r="AN46" s="44"/>
     </row>
     <row r="47" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
@@ -30586,7 +31645,7 @@
       <c r="G47" s="18"/>
       <c r="H47" s="18"/>
       <c r="I47" s="18"/>
-      <c r="J47" s="56"/>
+      <c r="J47" s="9"/>
       <c r="L47" s="2"/>
       <c r="M47" s="1"/>
       <c r="T47" s="1"/>
@@ -30609,25 +31668,25 @@
       <c r="AB47" s="35"/>
       <c r="AC47" s="35"/>
       <c r="AD47" s="35"/>
-      <c r="AF47" s="50"/>
-      <c r="AG47" s="50" t="s">
+      <c r="AF47" s="47"/>
+      <c r="AG47" s="47" t="s">
         <v>49</v>
       </c>
-      <c r="AH47" s="50" t="s">
+      <c r="AH47" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="AI47" s="50" t="s">
+      <c r="AI47" s="47" t="s">
         <v>50</v>
       </c>
-      <c r="AJ47" s="50" t="s">
+      <c r="AJ47" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="AK47" s="50" t="s">
+      <c r="AK47" s="47" t="s">
         <v>52</v>
       </c>
-      <c r="AL47" s="47"/>
-      <c r="AM47" s="47"/>
-      <c r="AN47" s="47"/>
+      <c r="AL47" s="44"/>
+      <c r="AM47" s="44"/>
+      <c r="AN47" s="44"/>
     </row>
     <row r="48" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
@@ -30647,52 +31706,52 @@
       <c r="G48" s="18"/>
       <c r="H48" s="18"/>
       <c r="I48" s="18"/>
-      <c r="J48" s="56"/>
+      <c r="J48" s="9"/>
       <c r="L48" s="2"/>
       <c r="M48" s="1"/>
       <c r="T48" s="1"/>
-      <c r="V48" s="45" t="s">
+      <c r="V48" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="W48" s="45">
+      <c r="W48" s="35">
         <v>2</v>
       </c>
-      <c r="X48" s="45">
+      <c r="X48" s="35">
         <v>1.0404378971357675E-2</v>
       </c>
-      <c r="Y48" s="45">
+      <c r="Y48" s="35">
         <v>5.2021894856788377E-3</v>
       </c>
-      <c r="Z48" s="45">
+      <c r="Z48" s="35">
         <v>3.8069678418784658</v>
       </c>
-      <c r="AA48" s="45">
+      <c r="AA48" s="35">
         <v>7.6060288642534488E-2</v>
       </c>
       <c r="AB48" s="35"/>
       <c r="AC48" s="35"/>
       <c r="AD48" s="35"/>
-      <c r="AF48" s="47" t="s">
+      <c r="AF48" s="44" t="s">
         <v>45</v>
       </c>
-      <c r="AG48" s="47">
+      <c r="AG48" s="44">
         <v>2</v>
       </c>
-      <c r="AH48" s="47">
+      <c r="AH48" s="44">
         <v>0.29280509096680318</v>
       </c>
-      <c r="AI48" s="47">
+      <c r="AI48" s="44">
         <v>0.14640254548340159</v>
       </c>
-      <c r="AJ48" s="47">
+      <c r="AJ48" s="44">
         <v>7.0090941756837504</v>
       </c>
-      <c r="AK48" s="47">
+      <c r="AK48" s="44">
         <v>2.1318648130072754E-2</v>
       </c>
-      <c r="AL48" s="47"/>
-      <c r="AM48" s="47"/>
-      <c r="AN48" s="47"/>
+      <c r="AL48" s="44"/>
+      <c r="AM48" s="44"/>
+      <c r="AN48" s="44"/>
     </row>
     <row r="49" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
@@ -30712,44 +31771,44 @@
       <c r="G49" s="18"/>
       <c r="H49" s="18"/>
       <c r="I49" s="18"/>
-      <c r="J49" s="56"/>
+      <c r="J49" s="9"/>
       <c r="L49" s="2"/>
       <c r="M49" s="1"/>
       <c r="T49" s="1"/>
-      <c r="V49" s="45" t="s">
+      <c r="V49" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="W49" s="45">
+      <c r="W49" s="35">
         <v>7</v>
       </c>
-      <c r="X49" s="45">
+      <c r="X49" s="35">
         <v>9.5654410313546299E-3</v>
       </c>
-      <c r="Y49" s="45">
+      <c r="Y49" s="35">
         <v>1.3664915759078044E-3</v>
       </c>
-      <c r="Z49" s="45"/>
-      <c r="AA49" s="45"/>
+      <c r="Z49" s="35"/>
+      <c r="AA49" s="35"/>
       <c r="AB49" s="35"/>
       <c r="AC49" s="35"/>
       <c r="AD49" s="35"/>
-      <c r="AF49" s="47" t="s">
+      <c r="AF49" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="AG49" s="47">
+      <c r="AG49" s="44">
         <v>7</v>
       </c>
-      <c r="AH49" s="47">
+      <c r="AH49" s="44">
         <v>0.14621259077088064</v>
       </c>
-      <c r="AI49" s="47">
+      <c r="AI49" s="44">
         <v>2.0887512967268661E-2</v>
       </c>
-      <c r="AJ49" s="47"/>
-      <c r="AK49" s="47"/>
-      <c r="AL49" s="47"/>
-      <c r="AM49" s="47"/>
-      <c r="AN49" s="47"/>
+      <c r="AJ49" s="44"/>
+      <c r="AK49" s="44"/>
+      <c r="AL49" s="44"/>
+      <c r="AM49" s="44"/>
+      <c r="AN49" s="44"/>
     </row>
     <row r="50" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="15" t="s">
@@ -30786,36 +31845,36 @@
       <c r="L50" s="2"/>
       <c r="M50" s="1"/>
       <c r="T50" s="1"/>
-      <c r="V50" s="46" t="s">
+      <c r="V50" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="W50" s="46">
+      <c r="W50" s="43">
         <v>9</v>
       </c>
-      <c r="X50" s="46">
+      <c r="X50" s="43">
         <v>1.9969820002712305E-2</v>
       </c>
-      <c r="Y50" s="46"/>
-      <c r="Z50" s="46"/>
-      <c r="AA50" s="46"/>
+      <c r="Y50" s="43"/>
+      <c r="Z50" s="43"/>
+      <c r="AA50" s="43"/>
       <c r="AB50" s="35"/>
       <c r="AC50" s="35"/>
       <c r="AD50" s="35"/>
-      <c r="AF50" s="49" t="s">
+      <c r="AF50" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="AG50" s="49">
+      <c r="AG50" s="46">
         <v>9</v>
       </c>
-      <c r="AH50" s="49">
+      <c r="AH50" s="46">
         <v>0.43901768173768385</v>
       </c>
-      <c r="AI50" s="49"/>
-      <c r="AJ50" s="49"/>
-      <c r="AK50" s="49"/>
-      <c r="AL50" s="47"/>
-      <c r="AM50" s="47"/>
-      <c r="AN50" s="47"/>
+      <c r="AI50" s="46"/>
+      <c r="AJ50" s="46"/>
+      <c r="AK50" s="46"/>
+      <c r="AL50" s="44"/>
+      <c r="AM50" s="44"/>
+      <c r="AN50" s="44"/>
     </row>
     <row r="51" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="15" t="s">
@@ -30835,7 +31894,7 @@
       <c r="G51" s="18"/>
       <c r="H51" s="18"/>
       <c r="I51" s="18"/>
-      <c r="J51" s="56"/>
+      <c r="J51" s="9"/>
       <c r="L51" s="2"/>
       <c r="M51" s="1"/>
       <c r="T51" s="1"/>
@@ -30848,15 +31907,15 @@
       <c r="AB51" s="35"/>
       <c r="AC51" s="35"/>
       <c r="AD51" s="35"/>
-      <c r="AF51" s="47"/>
-      <c r="AG51" s="47"/>
-      <c r="AH51" s="47"/>
-      <c r="AI51" s="47"/>
-      <c r="AJ51" s="47"/>
-      <c r="AK51" s="47"/>
-      <c r="AL51" s="47"/>
-      <c r="AM51" s="47"/>
-      <c r="AN51" s="47"/>
+      <c r="AF51" s="44"/>
+      <c r="AG51" s="44"/>
+      <c r="AH51" s="44"/>
+      <c r="AI51" s="44"/>
+      <c r="AJ51" s="44"/>
+      <c r="AK51" s="44"/>
+      <c r="AL51" s="44"/>
+      <c r="AM51" s="44"/>
+      <c r="AN51" s="44"/>
     </row>
     <row r="52" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
@@ -30878,7 +31937,7 @@
         <v>115.360934813333</v>
       </c>
       <c r="G52" s="18">
-        <f t="shared" ref="G51:G57" si="2">F52/C52</f>
+        <f t="shared" ref="G52:G57" si="2">F52/C52</f>
         <v>1.0331150820718804</v>
       </c>
       <c r="H52" s="18">
@@ -30918,29 +31977,29 @@
       <c r="AD52" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="AF52" s="50"/>
-      <c r="AG52" s="50" t="s">
+      <c r="AF52" s="47"/>
+      <c r="AG52" s="47" t="s">
         <v>53</v>
       </c>
-      <c r="AH52" s="50" t="s">
+      <c r="AH52" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="AI52" s="50" t="s">
+      <c r="AI52" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="AJ52" s="50" t="s">
+      <c r="AJ52" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="AK52" s="50" t="s">
+      <c r="AK52" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="AL52" s="50" t="s">
+      <c r="AL52" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="AM52" s="50" t="s">
+      <c r="AM52" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="AN52" s="50" t="s">
+      <c r="AN52" s="47" t="s">
         <v>59</v>
       </c>
     </row>
@@ -30964,7 +32023,7 @@
         <v>118.05576815000001</v>
       </c>
       <c r="G53" s="18">
-        <f t="shared" si="2"/>
+        <f>F53/C53</f>
         <v>1.0275460447393339</v>
       </c>
       <c r="H53" s="18">
@@ -30979,58 +32038,58 @@
       <c r="L53" s="2"/>
       <c r="M53" s="1"/>
       <c r="T53" s="1"/>
-      <c r="V53" s="45" t="s">
+      <c r="V53" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="W53" s="45">
+      <c r="W53" s="35">
         <v>-1.2574616091818591E-2</v>
       </c>
-      <c r="X53" s="45">
+      <c r="X53" s="35">
         <v>0.26302514322158932</v>
       </c>
-      <c r="Y53" s="45">
+      <c r="Y53" s="35">
         <v>-4.7807657997261978E-2</v>
       </c>
-      <c r="Z53" s="42">
+      <c r="Z53" s="41">
         <v>0.96320493852416367</v>
       </c>
-      <c r="AA53" s="45">
+      <c r="AA53" s="35">
         <v>-0.63453024853225437</v>
       </c>
-      <c r="AB53" s="45">
+      <c r="AB53" s="35">
         <v>0.60938101634861708</v>
       </c>
-      <c r="AC53" s="45">
+      <c r="AC53" s="35">
         <v>-0.63453024853225437</v>
       </c>
-      <c r="AD53" s="45">
+      <c r="AD53" s="35">
         <v>0.60938101634861708</v>
       </c>
-      <c r="AF53" s="47" t="s">
+      <c r="AF53" s="44" t="s">
         <v>48</v>
       </c>
-      <c r="AG53" s="47">
+      <c r="AG53" s="44">
         <v>1.4361728029697169</v>
       </c>
-      <c r="AH53" s="47">
+      <c r="AH53" s="44">
         <v>0.93644034793985709</v>
       </c>
-      <c r="AI53" s="47">
+      <c r="AI53" s="44">
         <v>1.5336511355253513</v>
       </c>
-      <c r="AJ53" s="51">
+      <c r="AJ53" s="48">
         <v>0.1689841959294115</v>
       </c>
-      <c r="AK53" s="47">
+      <c r="AK53" s="44">
         <v>-0.77815675393885453</v>
       </c>
-      <c r="AL53" s="47">
+      <c r="AL53" s="44">
         <v>3.6505023598782884</v>
       </c>
-      <c r="AM53" s="47">
+      <c r="AM53" s="44">
         <v>-0.77815675393885453</v>
       </c>
-      <c r="AN53" s="47">
+      <c r="AN53" s="44">
         <v>3.6505023598782884</v>
       </c>
     </row>
@@ -31069,58 +32128,58 @@
       <c r="L54" s="2"/>
       <c r="M54" s="1"/>
       <c r="T54" s="1"/>
-      <c r="V54" s="45" t="s">
+      <c r="V54" s="35" t="s">
         <v>63</v>
       </c>
-      <c r="W54" s="45">
+      <c r="W54" s="35">
         <v>0.14514560486276945</v>
       </c>
-      <c r="X54" s="45">
+      <c r="X54" s="35">
         <v>0.24897946993315845</v>
       </c>
-      <c r="Y54" s="45">
+      <c r="Y54" s="35">
         <v>0.58296214102205113</v>
       </c>
-      <c r="Z54" s="42">
+      <c r="Z54" s="41">
         <v>0.57820722298127447</v>
       </c>
-      <c r="AA54" s="45">
+      <c r="AA54" s="35">
         <v>-0.44359728788989367</v>
       </c>
-      <c r="AB54" s="45">
+      <c r="AB54" s="35">
         <v>0.73388849761543251</v>
       </c>
-      <c r="AC54" s="45">
+      <c r="AC54" s="35">
         <v>-0.44359728788989367</v>
       </c>
-      <c r="AD54" s="45">
+      <c r="AD54" s="35">
         <v>0.73388849761543251</v>
       </c>
-      <c r="AF54" s="47" t="s">
+      <c r="AF54" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="AG54" s="47">
+      <c r="AG54" s="44">
         <v>-1.7036514188702609</v>
       </c>
-      <c r="AH54" s="47">
+      <c r="AH54" s="44">
         <v>0.89368571318009815</v>
       </c>
-      <c r="AI54" s="47">
+      <c r="AI54" s="44">
         <v>-1.9063205260470983</v>
       </c>
-      <c r="AJ54" s="51">
+      <c r="AJ54" s="48">
         <v>9.8288110769124692E-2</v>
       </c>
-      <c r="AK54" s="47">
+      <c r="AK54" s="44">
         <v>-3.8168823295579148</v>
       </c>
-      <c r="AL54" s="47">
+      <c r="AL54" s="44">
         <v>0.40957949181739295</v>
       </c>
-      <c r="AM54" s="47">
+      <c r="AM54" s="44">
         <v>-3.8168823295579148</v>
       </c>
-      <c r="AN54" s="47">
+      <c r="AN54" s="44">
         <v>0.40957949181739295</v>
       </c>
     </row>
@@ -31166,58 +32225,58 @@
       <c r="R55" s="1"/>
       <c r="S55" s="1"/>
       <c r="T55" s="1"/>
-      <c r="V55" s="46" t="s">
+      <c r="V55" s="43" t="s">
         <v>33</v>
       </c>
-      <c r="W55" s="46">
+      <c r="W55" s="43">
         <v>9.2100179192589095E-3</v>
       </c>
-      <c r="X55" s="46">
+      <c r="X55" s="43">
         <v>3.5136946825407508E-3</v>
       </c>
-      <c r="Y55" s="46">
+      <c r="Y55" s="43">
         <v>2.6211776353314655</v>
       </c>
-      <c r="Z55" s="43">
+      <c r="Z55" s="42">
         <v>3.4350324161060167E-2</v>
       </c>
-      <c r="AA55" s="46">
+      <c r="AA55" s="43">
         <v>9.0145026023043945E-4</v>
       </c>
-      <c r="AB55" s="46">
+      <c r="AB55" s="43">
         <v>1.751858557828738E-2</v>
       </c>
-      <c r="AC55" s="46">
+      <c r="AC55" s="43">
         <v>9.0145026023043945E-4</v>
       </c>
-      <c r="AD55" s="46">
+      <c r="AD55" s="43">
         <v>1.751858557828738E-2</v>
       </c>
-      <c r="AF55" s="49" t="s">
+      <c r="AF55" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="AG55" s="49">
+      <c r="AG55" s="46">
         <v>-4.8419684545285259E-2</v>
       </c>
-      <c r="AH55" s="49">
+      <c r="AH55" s="46">
         <v>1.385503060115428E-2</v>
       </c>
-      <c r="AI55" s="49">
+      <c r="AI55" s="46">
         <v>-3.4947367450239595</v>
       </c>
-      <c r="AJ55" s="53">
+      <c r="AJ55" s="49">
         <v>1.0064173436446097E-2</v>
       </c>
-      <c r="AK55" s="49">
+      <c r="AK55" s="46">
         <v>-8.118162591133482E-2</v>
       </c>
-      <c r="AL55" s="49">
+      <c r="AL55" s="46">
         <v>-1.5657743179235691E-2</v>
       </c>
-      <c r="AM55" s="49">
+      <c r="AM55" s="46">
         <v>-8.118162591133482E-2</v>
       </c>
-      <c r="AN55" s="49">
+      <c r="AN55" s="46">
         <v>-1.5657743179235691E-2</v>
       </c>
     </row>
@@ -31335,7 +32394,7 @@
       <c r="I60" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="J60" s="54"/>
+      <c r="J60" s="37"/>
     </row>
     <row r="61" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A61" s="15" t="s">
@@ -31353,7 +32412,7 @@
       <c r="G61" s="18"/>
       <c r="H61" s="25"/>
       <c r="I61" s="15"/>
-      <c r="J61" s="55"/>
+      <c r="J61" s="1"/>
     </row>
     <row r="62" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
@@ -31375,7 +32434,7 @@
         <v>71.117321599999997</v>
       </c>
       <c r="G62" s="18">
-        <v>1.1737788669959499</v>
+        <v>1.1737788669959504</v>
       </c>
       <c r="H62" s="18">
         <v>4</v>
@@ -31407,7 +32466,7 @@
         <v>74.728308609999999</v>
       </c>
       <c r="G63" s="18">
-        <v>1.01827696825768</v>
+        <v>1.0182769682576838</v>
       </c>
       <c r="H63" s="18">
         <v>1.1385255280790201</v>
@@ -31469,7 +32528,7 @@
       <c r="G65" s="18"/>
       <c r="H65" s="18"/>
       <c r="I65" s="18"/>
-      <c r="J65" s="56"/>
+      <c r="J65" s="9"/>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="15" t="s">
@@ -31489,7 +32548,7 @@
       <c r="G66" s="18"/>
       <c r="H66" s="18"/>
       <c r="I66" s="18"/>
-      <c r="J66" s="56"/>
+      <c r="J66" s="9"/>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="15" t="s">
@@ -31509,7 +32568,7 @@
       <c r="G67" s="18"/>
       <c r="H67" s="18"/>
       <c r="I67" s="18"/>
-      <c r="J67" s="56"/>
+      <c r="J67" s="9"/>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="15" t="s">
@@ -31529,7 +32588,7 @@
       <c r="G68" s="18"/>
       <c r="H68" s="18"/>
       <c r="I68" s="18"/>
-      <c r="J68" s="56"/>
+      <c r="J68" s="9"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="15" t="s">
@@ -31551,7 +32610,6 @@
         <v>115.079453056666</v>
       </c>
       <c r="G69" s="18">
-        <f>F69/C69</f>
         <v>1.0393698938576728</v>
       </c>
       <c r="H69" s="18">
@@ -31582,7 +32640,7 @@
       <c r="G70" s="18"/>
       <c r="H70" s="18"/>
       <c r="I70" s="18"/>
-      <c r="J70" s="56"/>
+      <c r="J70" s="9"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="15" t="s">
@@ -31604,7 +32662,7 @@
         <v>115.360934813333</v>
       </c>
       <c r="G71" s="17">
-        <v>1.0311456359907301</v>
+        <v>1.0331150820718804</v>
       </c>
       <c r="H71" s="18">
         <v>19.594840851392899</v>
@@ -31636,7 +32694,7 @@
         <v>118.05576815000001</v>
       </c>
       <c r="G72" s="17">
-        <v>1.0328896319418399</v>
+        <v>1.0275460447393339</v>
       </c>
       <c r="H72" s="18">
         <v>17.2552427011953</v>
@@ -31668,7 +32726,7 @@
         <v>119.77022043333299</v>
       </c>
       <c r="G73" s="17">
-        <v>1.0327006459464001</v>
+        <v>1.0275826446035865</v>
       </c>
       <c r="H73" s="18">
         <v>17.024424898784201</v>
@@ -31700,7 +32758,7 @@
         <v>125.17995179</v>
       </c>
       <c r="G74" s="17">
-        <v>1.06939420314209</v>
+        <v>1.0396485920727681</v>
       </c>
       <c r="H74" s="18">
         <v>15.1069524712688</v>
@@ -31732,7 +32790,7 @@
         <v>128.631154973333</v>
       </c>
       <c r="G75" s="17">
-        <v>1.12591121276406</v>
+        <v>1.0831630031367767</v>
       </c>
       <c r="H75" s="18">
         <v>21.9579587943592</v>
@@ -31764,7 +32822,7 @@
         <v>127.417386873333</v>
       </c>
       <c r="G76" s="17">
-        <v>1.06457347177821</v>
+        <v>1.0183454205725238</v>
       </c>
       <c r="H76" s="18">
         <v>16.640165980770899</v>

</xml_diff>